<commit_message>
Checkpoint: SeriesA and SeriesB cap tables fixed
</commit_message>
<xml_diff>
--- a/runs/20260414-101230/models/model.xlsx
+++ b/runs/20260414-101230/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{697DD009-A20A-EF49-90B3-0FDB66A0933D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B600FD6-D3CE-704C-AE21-85E9774F5956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="__temp__" sheetId="103" r:id="rId1"/>
-    <sheet name="SidekickCapTable" sheetId="111" r:id="rId2"/>
-    <sheet name="Inputs" sheetId="112" r:id="rId3"/>
+    <sheet name="SidekickCapTable" sheetId="111" r:id="rId1"/>
+    <sheet name="Inputs" sheetId="112" r:id="rId2"/>
+    <sheet name="SeriesA" sheetId="113" r:id="rId3"/>
+    <sheet name="SeriesB" sheetId="114" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="121">
   <si>
     <t>Total</t>
   </si>
@@ -196,12 +197,63 @@
     <t>SAFE Investments</t>
   </si>
   <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t>Pre A</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>1011 Ventures</t>
+  </si>
+  <si>
     <t>Other Series A Investors</t>
   </si>
   <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
     <t>Pre-Money Valuation</t>
   </si>
   <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
     <t>1011 Ventures Investment</t>
   </si>
   <si>
@@ -211,9 +263,39 @@
     <t>SAFE Post-Money Valuation Cap</t>
   </si>
   <si>
+    <t>Series B</t>
+  </si>
+  <si>
+    <t>Pre B</t>
+  </si>
+  <si>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>Option</t>
+  </si>
+  <si>
+    <t>Other Common Shareholders</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other SAFE Investors</t>
+  </si>
+  <si>
+    <t>Other Series B Investors</t>
+  </si>
+  <si>
+    <t>Invested</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
   <si>
+    <t>SIDEKICK &amp; 1011 VENTURES SERIES A</t>
+  </si>
+  <si>
     <t>Sidekick (Think More Security, Inc.)</t>
   </si>
   <si>
@@ -275,18 +357,61 @@
   </si>
   <si>
     <t>Assumed Exit Date (Post-B)</t>
+  </si>
+  <si>
+    <t>Safe Preferred</t>
+  </si>
+  <si>
+    <t>Series A Preferred</t>
+  </si>
+  <si>
+    <t>Safe Pref</t>
+  </si>
+  <si>
+    <t>ESOP Issued and Outstanding</t>
+  </si>
+  <si>
+    <t>Safe Price</t>
+  </si>
+  <si>
+    <t>Series A Price</t>
+  </si>
+  <si>
+    <t>SIDEKICK &amp; 1011 VENTURES SERIES B</t>
+  </si>
+  <si>
+    <t>Series B Preferred</t>
+  </si>
+  <si>
+    <t>Total Cap</t>
+  </si>
+  <si>
+    <t>ESOP Available (from Series A)</t>
+  </si>
+  <si>
+    <t>ESOP Gross Top-Up (Series B)</t>
+  </si>
+  <si>
+    <t>Series B Price</t>
+  </si>
+  <si>
+    <t>Safe Price (from Series A)</t>
+  </si>
+  <si>
+    <t>Series A Price (from Series A)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -437,6 +562,12 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
       <name val="Garamond"/>
       <family val="1"/>
     </font>
@@ -648,7 +779,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -763,6 +894,88 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -808,7 +1021,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -821,29 +1034,97 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="5" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="5" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1236,16 +1517,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D555A474-5AC6-5048-8F91-0C2401531367}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD337B6E-AF57-924A-818B-D8F76BC5BE6B}">
   <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1288,7 +1559,7 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="I2" s="3"/>
@@ -1301,25 +1572,25 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="16" t="s">
         <v>7</v>
       </c>
       <c r="I3" s="3"/>
@@ -1332,20 +1603,20 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="17">
         <v>3600000</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10">
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="18">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
@@ -1359,20 +1630,20 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="17">
         <v>3600000</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10">
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="18">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
@@ -1386,20 +1657,20 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="17">
         <v>222187</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10">
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="18">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
@@ -1413,20 +1684,20 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="17">
         <v>592500</v>
       </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10">
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="18">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
@@ -1440,20 +1711,20 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="17">
         <v>592500</v>
       </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10">
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="18">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
@@ -1467,22 +1738,22 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="17">
         <v>13500</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="17">
         <v>98900</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10">
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="18">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
@@ -1496,20 +1767,20 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="17">
         <v>9000</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10">
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="18">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
@@ -1523,20 +1794,20 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10">
+      <c r="C11" s="17"/>
+      <c r="D11" s="17">
         <v>95000</v>
       </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10">
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="18">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
@@ -1550,20 +1821,20 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17">
         <v>25000</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10">
+      <c r="F12" s="17"/>
+      <c r="G12" s="17">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="18">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
@@ -1577,20 +1848,20 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17">
         <v>41562</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10">
+      <c r="F13" s="17"/>
+      <c r="G13" s="17">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="18">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
@@ -1604,20 +1875,20 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17">
         <v>285000</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10">
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="18">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
@@ -1631,20 +1902,20 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17">
         <v>50000</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10">
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="18">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
@@ -1658,20 +1929,20 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10">
+      <c r="C16" s="17"/>
+      <c r="D16" s="17">
         <v>285000</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10">
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="18">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
@@ -1685,20 +1956,20 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10">
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17">
         <v>96186</v>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10">
+      <c r="F17" s="17"/>
+      <c r="G17" s="17">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="18">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
@@ -1712,20 +1983,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10">
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17">
         <v>48095</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10">
+      <c r="F18" s="17"/>
+      <c r="G18" s="17">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="18">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
@@ -1739,20 +2010,20 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17">
         <v>12395</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="17">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="11">
+      <c r="H19" s="18">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
@@ -1766,20 +2037,20 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17">
         <v>8333</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="17">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="11">
+      <c r="H20" s="18">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
@@ -1793,20 +2064,20 @@
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17">
         <v>65105</v>
       </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10">
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="11">
+      <c r="H21" s="18">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
@@ -1837,26 +2108,26 @@
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="17">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="17">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="17">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="17">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="17">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
@@ -1905,7 +2176,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="16" t="s">
         <v>52</v>
       </c>
       <c r="C26" s="3"/>
@@ -1924,14 +2195,14 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9" t="s">
+      <c r="D27" s="16"/>
+      <c r="E27" s="16" t="s">
         <v>27</v>
       </c>
       <c r="F27" s="3"/>
@@ -1947,14 +2218,14 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="19">
         <v>25000</v>
       </c>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8" t="s">
+      <c r="D28" s="15"/>
+      <c r="E28" s="15" t="s">
         <v>28</v>
       </c>
       <c r="F28" s="3"/>
@@ -1970,14 +2241,14 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="19">
         <v>25000</v>
       </c>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
@@ -1991,14 +2262,14 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="19">
         <v>137170.75</v>
       </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -2012,14 +2283,14 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="19">
         <v>3846829.25</v>
       </c>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
@@ -2033,15 +2304,15 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="19">
         <v>16566</v>
       </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8" t="s">
-        <v>58</v>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -2056,14 +2327,14 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="19">
         <v>250000</v>
       </c>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
@@ -2077,14 +2348,14 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="19">
         <v>100000</v>
       </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
@@ -2098,14 +2369,14 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="19">
         <v>300000</v>
       </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8" t="s">
+      <c r="D35" s="15"/>
+      <c r="E35" s="15" t="s">
         <v>28</v>
       </c>
       <c r="F35" s="3"/>
@@ -2121,14 +2392,14 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="19">
         <v>37500</v>
       </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8" t="s">
+      <c r="D36" s="15"/>
+      <c r="E36" s="15" t="s">
         <v>36</v>
       </c>
       <c r="F36" s="3"/>
@@ -2144,14 +2415,14 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="19">
         <v>250000</v>
       </c>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
@@ -2165,14 +2436,14 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="19">
         <v>100000</v>
       </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
@@ -2186,15 +2457,15 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="19">
         <v>41164</v>
       </c>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8" t="s">
-        <v>58</v>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -2209,15 +2480,15 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="19">
         <v>2328778</v>
       </c>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8" t="s">
-        <v>58</v>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -2232,14 +2503,14 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="19">
         <v>1506000</v>
       </c>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8" t="s">
+      <c r="D41" s="15"/>
+      <c r="E41" s="15" t="s">
         <v>42</v>
       </c>
       <c r="F41" s="3"/>
@@ -2255,14 +2526,14 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="19">
         <v>50000</v>
       </c>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
@@ -2276,14 +2547,14 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="3"/>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="19">
         <v>212500</v>
       </c>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8" t="s">
+      <c r="D43" s="15"/>
+      <c r="E43" s="15" t="s">
         <v>36</v>
       </c>
       <c r="F43" s="3"/>
@@ -2299,14 +2570,14 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C44" s="12">
+      <c r="C44" s="19">
         <v>25000</v>
       </c>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
@@ -2320,15 +2591,15 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="19">
         <v>61746</v>
       </c>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8" t="s">
-        <v>58</v>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -2343,14 +2614,14 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" s="3"/>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="12">
+      <c r="C46" s="19">
         <v>100000</v>
       </c>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
@@ -2364,14 +2635,14 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" s="3"/>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C47" s="12">
+      <c r="C47" s="19">
         <v>100000</v>
       </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
@@ -2385,15 +2656,15 @@
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" s="3"/>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C48" s="12">
+      <c r="C48" s="19">
         <v>61746</v>
       </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8" t="s">
-        <v>58</v>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -2408,14 +2679,14 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" s="3"/>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="12">
+      <c r="C49" s="19">
         <v>250000</v>
       </c>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8" t="s">
+      <c r="D49" s="15"/>
+      <c r="E49" s="15" t="s">
         <v>51</v>
       </c>
       <c r="F49" s="3"/>
@@ -2447,10 +2718,10 @@
       <c r="O50" s="3"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C51" s="14">
+      <c r="C51" s="26">
         <f>SUM(C28:C49)</f>
         <v>9825000</v>
       </c>
@@ -2460,7 +2731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EE5CF8-CE71-224D-8F1F-D43A309B5A51}">
   <dimension ref="B1:C33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2472,200 +2743,1755 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B1" s="13" t="s">
-        <v>59</v>
+      <c r="B1" s="20" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B2" s="13" t="s">
-        <v>60</v>
+      <c r="B2" s="20" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="15">
+        <v>70</v>
+      </c>
+      <c r="C5" s="27">
         <v>60000000</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="15">
+        <v>89</v>
+      </c>
+      <c r="C6" s="27">
         <v>20000000</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="15">
+        <v>72</v>
+      </c>
+      <c r="C7" s="27">
         <v>12000000</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="15">
+        <v>73</v>
+      </c>
+      <c r="C8" s="27">
         <v>5000000</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="15">
+        <v>67</v>
+      </c>
+      <c r="C9" s="27">
         <v>3000000</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="16">
+        <v>90</v>
+      </c>
+      <c r="C10" s="28">
         <f>C6-(C7+C8+C9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="15">
+        <v>74</v>
+      </c>
+      <c r="C13" s="27">
         <v>50000000</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="5" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C16" s="6">
+        <v>93</v>
+      </c>
+      <c r="C16" s="7">
         <v>0.1</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
-        <v>67</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="15">
+        <v>70</v>
+      </c>
+      <c r="C19" s="27">
         <v>150000000</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" s="15">
+        <v>95</v>
+      </c>
+      <c r="C20" s="27">
         <v>30000000</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="15">
+        <v>96</v>
+      </c>
+      <c r="C21" s="27">
         <v>15000000</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C22" s="15">
+        <v>97</v>
+      </c>
+      <c r="C22" s="27">
         <v>15000000</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="6">
+        <v>98</v>
+      </c>
+      <c r="C23" s="7">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B26" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" s="6">
+        <v>100</v>
+      </c>
+      <c r="C26" s="7">
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C27" s="6">
+        <v>101</v>
+      </c>
+      <c r="C27" s="7">
         <v>0.1</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C30" s="17">
+        <v>103</v>
+      </c>
+      <c r="C30" s="29">
         <v>46174</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C31" s="17">
+        <v>104</v>
+      </c>
+      <c r="C31" s="29">
         <f>DATE(YEAR(C30)+1,MONTH(C30)+6,DAY(C30))</f>
         <v>46722</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C32" s="18">
+        <v>105</v>
+      </c>
+      <c r="C32" s="30">
         <f>DATE(YEAR(C30)+5,MONTH(C30),DAY(C30))</f>
         <v>48000</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C33" s="18">
+        <v>106</v>
+      </c>
+      <c r="C33" s="30">
         <f>DATE(YEAR(C31)+3,MONTH(C31),DAY(C31))</f>
         <v>47818</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C11AFC32-5C18-724D-B91B-63EE81C382F3}">
+  <dimension ref="B1:O25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.5" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="16.33203125" customWidth="1"/>
+    <col min="11" max="11" width="0.6640625" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.6640625" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="8.83203125" customWidth="1"/>
+    <col min="16" max="16" width="7.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+    </row>
+    <row r="2" spans="2:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+    </row>
+    <row r="3" spans="2:15" ht="16.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="G4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="L4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="6"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="C5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B7" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="31"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B8" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="8">
+        <f>SidekickCapTable!C4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="9">
+        <f>C8+E8+G8+J8</f>
+        <v>3600000</v>
+      </c>
+      <c r="O8" s="32">
+        <f ca="1">N8/$N$20</f>
+        <v>0.20126781328857071</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B9" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8">
+        <f>SidekickCapTable!C5</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="9">
+        <f>C9+E9+G9+J9</f>
+        <v>3600000</v>
+      </c>
+      <c r="O9" s="32">
+        <f ca="1">N9/$N$20</f>
+        <v>0.20126781328857071</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B10" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="8">
+        <f>SUM(SidekickCapTable!C6:C10)</f>
+        <v>1429687</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="9">
+        <f>C10+E10+G10+J10</f>
+        <v>1429687</v>
+      </c>
+      <c r="O10" s="32">
+        <f ca="1">N10/$N$20</f>
+        <v>7.9930548938082435E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B11" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="8">
+        <f>SUM(SidekickCapTable!D4:D21,SidekickCapTable!E4:E21,SidekickCapTable!F4:F21)-SidekickCapTable!D21</f>
+        <v>1045471</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="9">
+        <f>C11+E11+G11+J11</f>
+        <v>1045471</v>
+      </c>
+      <c r="O11" s="32">
+        <f ca="1">N11/$N$20</f>
+        <v>5.8449906118504251E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B12" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="1">
+        <f>SidekickCapTable!D21</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="8">
+        <f ca="1">Inputs!C16*N20-C12</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="9">
+        <f ca="1">C12+G12</f>
+        <v>1788661.5555555557</v>
+      </c>
+      <c r="O12" s="32">
+        <f ca="1">N12/$N$20</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B13" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="43">
+        <f>SUM(C8:C12)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="43">
+        <f ca="1">G12</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="35"/>
+      <c r="M13" s="35"/>
+      <c r="N13" s="34">
+        <f ca="1">SUM(N8:N12)</f>
+        <v>11463819.555555556</v>
+      </c>
+      <c r="O13" s="36">
+        <f ca="1">N13/$N$20</f>
+        <v>0.64091608163372815</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B14" s="24"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="33"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="33"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B16" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="11">
+        <f>SUM(SidekickCapTable!C30,SidekickCapTable!C31,SidekickCapTable!C32,SidekickCapTable!C39,SidekickCapTable!C40,SidekickCapTable!C41,SidekickCapTable!C45,SidekickCapTable!C48)</f>
+        <v>8000000</v>
+      </c>
+      <c r="E16" s="9">
+        <f ca="1">IFERROR(ROUND(D16/N23,0),0)</f>
+        <v>1939567</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="10">
+        <f>Inputs!C8</f>
+        <v>5000000</v>
+      </c>
+      <c r="J16" s="9">
+        <f ca="1">IFERROR(ROUND(I16/N24,0),0)</f>
+        <v>1010191</v>
+      </c>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="9">
+        <f ca="1">C16+E16+J16</f>
+        <v>2949758</v>
+      </c>
+      <c r="O16" s="32">
+        <f ca="1">N16/$N$20</f>
+        <v>0.16491426177512994</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B17" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="11">
+        <f>SUM(SidekickCapTable!C28,SidekickCapTable!C29,SidekickCapTable!C33,SidekickCapTable!C34,SidekickCapTable!C35,SidekickCapTable!C36,SidekickCapTable!C37,SidekickCapTable!C38,SidekickCapTable!C42,SidekickCapTable!C43,SidekickCapTable!C44,SidekickCapTable!C46,SidekickCapTable!C47,SidekickCapTable!C49)</f>
+        <v>1825000</v>
+      </c>
+      <c r="E17" s="9">
+        <f ca="1">IFERROR(ROUND(D17/N23,0),0)</f>
+        <v>442464</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="9">
+        <f ca="1">C17+E17+J17</f>
+        <v>442464</v>
+      </c>
+      <c r="O17" s="32">
+        <f ca="1">N17/$N$20</f>
+        <v>2.4737156038587265E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B18" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="10">
+        <f>Inputs!C7</f>
+        <v>12000000</v>
+      </c>
+      <c r="J18" s="9">
+        <f ca="1">IFERROR(ROUND(I18/N24,0),0)</f>
+        <v>2424459</v>
+      </c>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="9">
+        <f ca="1">C18+E18+J18</f>
+        <v>2424459</v>
+      </c>
+      <c r="O18" s="32">
+        <f ca="1">N18/$N$20</f>
+        <v>0.13554598926049857</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B19" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="10">
+        <f>Inputs!C9</f>
+        <v>3000000</v>
+      </c>
+      <c r="J19" s="9">
+        <f ca="1">IFERROR(ROUND(I19/N24,0),0)</f>
+        <v>606115</v>
+      </c>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="9">
+        <f ca="1">C19+E19+J19</f>
+        <v>606115</v>
+      </c>
+      <c r="O19" s="32">
+        <f ca="1">N19/$N$20</f>
+        <v>3.3886511292056123E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="38">
+        <f>C13+SUM(C16:C19)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D20" s="39">
+        <f>SUM(D16:D19)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E20" s="38">
+        <f ca="1">SUM(E16:E19)</f>
+        <v>2382031</v>
+      </c>
+      <c r="F20" s="40"/>
+      <c r="G20" s="38">
+        <f ca="1">G13</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H20" s="40"/>
+      <c r="I20" s="39">
+        <f>SUM(I16:I19)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J20" s="38">
+        <f ca="1">SUM(J16:J19)</f>
+        <v>4040765</v>
+      </c>
+      <c r="K20" s="40"/>
+      <c r="L20" s="41">
+        <f>L12</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="40"/>
+      <c r="N20" s="38">
+        <f ca="1">SUM(N8:N12)+SUM(N16:N19)</f>
+        <v>17886615.555555556</v>
+      </c>
+      <c r="O20" s="42">
+        <f ca="1">SUM(O8:O12)+SUM(O16:O19)</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B22" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="13">
+        <f ca="1">Inputs!C13/(C8+C9+C10+C11+E16+E17+SidekickCapTable!D21)</f>
+        <v>4.1246318559836945</v>
+      </c>
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="13">
+        <f ca="1">Inputs!C5/(C8+C9+C10+C11+E16+E17+SidekickCapTable!D21)</f>
+        <v>4.9495582271804333</v>
+      </c>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B25" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="11">
+        <f>Inputs!C5+Inputs!C6</f>
+        <v>80000000</v>
+      </c>
+      <c r="O25" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31A13944-6939-5743-A643-DF5CE87713DB}">
+  <dimension ref="B1:T30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="33.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" customWidth="1"/>
+    <col min="8" max="8" width="0.6640625" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="0.6640625" customWidth="1"/>
+    <col min="12" max="12" width="11.33203125" customWidth="1"/>
+    <col min="13" max="13" width="0.6640625" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="16.33203125" customWidth="1"/>
+    <col min="16" max="16" width="0.6640625" customWidth="1"/>
+    <col min="17" max="17" width="11.33203125" customWidth="1"/>
+    <col min="18" max="18" width="0.6640625" customWidth="1"/>
+    <col min="19" max="19" width="15" customWidth="1"/>
+    <col min="20" max="20" width="8.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B1" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+    </row>
+    <row r="2" spans="2:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+    </row>
+    <row r="3" spans="2:20" ht="16.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:20" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="G4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="L4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O4" s="6"/>
+      <c r="Q4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="T4" s="6"/>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B7" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="31"/>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="31"/>
+      <c r="R7" s="31"/>
+      <c r="S7" s="31"/>
+      <c r="T7" s="31"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B8" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="8">
+        <f>SeriesA!C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="9">
+        <f>C8+E8+G8+J8+O8+Q8</f>
+        <v>3600000</v>
+      </c>
+      <c r="T8" s="32">
+        <f ca="1">S8/$S$23</f>
+        <v>0.15598255610610803</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B9" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8">
+        <f>SeriesA!C9</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="9">
+        <f>C9+E9+G9+J9+O9+Q9</f>
+        <v>3600000</v>
+      </c>
+      <c r="T9" s="32">
+        <f ca="1">S9/$S$23</f>
+        <v>0.15598255610610803</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B10" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="8">
+        <f>SeriesA!C10</f>
+        <v>1429687</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="9">
+        <f>C10+E10+G10+J10+O10+Q10</f>
+        <v>1429687</v>
+      </c>
+      <c r="T10" s="32">
+        <f ca="1">S10/$S$23</f>
+        <v>6.194617574768703E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B11" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="8">
+        <f>SeriesA!C11</f>
+        <v>1045471</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="9">
+        <f>C11+E11+G11+J11+O11+Q11</f>
+        <v>1045471</v>
+      </c>
+      <c r="T11" s="32">
+        <f ca="1">S11/$S$23</f>
+        <v>4.52986774763358E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B12" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="8">
+        <f>SeriesA!C12</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="8">
+        <f ca="1">SeriesA!G12</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="9">
+        <f ca="1">C12+E12+G12+J12+O12+Q12</f>
+        <v>1788661.5555555557</v>
+      </c>
+      <c r="T12" s="32">
+        <f ca="1">S12/$S$23</f>
+        <v>7.750000040118972E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B13" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="9">
+        <f ca="1">Inputs!C23*S23</f>
+        <v>1615565.2676224613</v>
+      </c>
+      <c r="R13" s="3"/>
+      <c r="S13" s="9">
+        <f ca="1">C13+E13+G13+J13+O13+Q13</f>
+        <v>1615565.2676224613</v>
+      </c>
+      <c r="T13" s="32">
+        <f ca="1">S13/$S$23</f>
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B14" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="43">
+        <f>SUM(C8:C13)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="43">
+        <f ca="1">G12</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="35"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="43">
+        <f ca="1">Q13</f>
+        <v>1615565.2676224613</v>
+      </c>
+      <c r="R14" s="35"/>
+      <c r="S14" s="34">
+        <f ca="1">SUM(S8:S13)</f>
+        <v>13079384.823178018</v>
+      </c>
+      <c r="T14" s="36">
+        <f ca="1">S14/$S$23</f>
+        <v>0.56670996583742872</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B15" s="24"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="33"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B16" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="33"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B17" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="10">
+        <f>SeriesA!D16</f>
+        <v>8000000</v>
+      </c>
+      <c r="E17" s="8">
+        <f ca="1">SeriesA!E16</f>
+        <v>1939567</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="10">
+        <f>SeriesA!I16</f>
+        <v>5000000</v>
+      </c>
+      <c r="J17" s="8">
+        <f ca="1">SeriesA!J16</f>
+        <v>1010191</v>
+      </c>
+      <c r="K17" s="3"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="11">
+        <f ca="1">Inputs!C22*(SeriesA!O16/(SeriesA!O16+SeriesA!O18+SeriesA!O19))</f>
+        <v>7398647.7673814772</v>
+      </c>
+      <c r="O17" s="9">
+        <f ca="1">IFERROR(ROUND(N17/$S$26,0),0)</f>
+        <v>882245</v>
+      </c>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="9">
+        <f ca="1">C17+E17+J17+O17</f>
+        <v>3832003</v>
+      </c>
+      <c r="T17" s="32">
+        <f ca="1">S17/$S$23</f>
+        <v>0.16603489526285398</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B18" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="10">
+        <f>SeriesA!D17</f>
+        <v>1825000</v>
+      </c>
+      <c r="E18" s="8">
+        <f ca="1">SeriesA!E17</f>
+        <v>442464</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="9">
+        <f ca="1">C18+E18+J18+O18</f>
+        <v>442464</v>
+      </c>
+      <c r="T18" s="32">
+        <f ca="1">S18/$S$23</f>
+        <v>1.9171296029148053E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B19" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="10">
+        <f>SeriesA!I18</f>
+        <v>12000000</v>
+      </c>
+      <c r="J19" s="8">
+        <f ca="1">SeriesA!J18</f>
+        <v>2424459</v>
+      </c>
+      <c r="K19" s="3"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="11">
+        <f ca="1">Inputs!C22*(SeriesA!O18/(SeriesA!O16+SeriesA!O18+SeriesA!O19))</f>
+        <v>6081081.2844504286</v>
+      </c>
+      <c r="O19" s="9">
+        <f ca="1">IFERROR(ROUND(N19/$S$26,0),0)</f>
+        <v>725133</v>
+      </c>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="9">
+        <f ca="1">C19+E19+J19+O19</f>
+        <v>3149592</v>
+      </c>
+      <c r="T19" s="32">
+        <f ca="1">S19/$S$23</f>
+        <v>0.13646705856981919</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B20" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="10">
+        <f>SeriesA!I19</f>
+        <v>3000000</v>
+      </c>
+      <c r="J20" s="8">
+        <f ca="1">SeriesA!J19</f>
+        <v>606115</v>
+      </c>
+      <c r="K20" s="3"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="11">
+        <f ca="1">Inputs!C22*(SeriesA!O19/(SeriesA!O16+SeriesA!O18+SeriesA!O19))</f>
+        <v>1520270.9481680952</v>
+      </c>
+      <c r="O20" s="9">
+        <f ca="1">IFERROR(ROUND(N20/$S$26,0),0)</f>
+        <v>181283</v>
+      </c>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="9">
+        <f ca="1">C20+E20+J20+O20</f>
+        <v>787398</v>
+      </c>
+      <c r="T20" s="32">
+        <f ca="1">S20/$S$23</f>
+        <v>3.4116764642454799E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B21" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="10">
+        <f>Inputs!C21</f>
+        <v>15000000</v>
+      </c>
+      <c r="O21" s="9">
+        <f ca="1">IFERROR(ROUND(N21/$S$26,0),0)</f>
+        <v>1788662</v>
+      </c>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="9">
+        <f ca="1">C21+E21+J21+O21</f>
+        <v>1788662</v>
+      </c>
+      <c r="T21" s="32">
+        <f ca="1">S21/$S$23</f>
+        <v>7.7500019658295394E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B22" s="24"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="33"/>
+    </row>
+    <row r="23" spans="2:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="38">
+        <f>C14+SUM(C17:C21)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D23" s="39">
+        <f>SUM(D17:D21)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E23" s="38">
+        <f ca="1">SUM(E17:E21)</f>
+        <v>2382031</v>
+      </c>
+      <c r="F23" s="40"/>
+      <c r="G23" s="38">
+        <f ca="1">G14</f>
+        <v>1723556.5555555557</v>
+      </c>
+      <c r="H23" s="40"/>
+      <c r="I23" s="39">
+        <f>SUM(I17:I21)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J23" s="38">
+        <f ca="1">SUM(J17:J21)</f>
+        <v>4040765</v>
+      </c>
+      <c r="K23" s="40"/>
+      <c r="L23" s="38">
+        <f>L12</f>
+        <v>0</v>
+      </c>
+      <c r="M23" s="40"/>
+      <c r="N23" s="39">
+        <f ca="1">SUM(N17:N21)</f>
+        <v>30000000</v>
+      </c>
+      <c r="O23" s="38">
+        <f ca="1">SUM(O17:O21)</f>
+        <v>3577323</v>
+      </c>
+      <c r="P23" s="40"/>
+      <c r="Q23" s="38">
+        <f ca="1">Q14</f>
+        <v>1615565.2676224613</v>
+      </c>
+      <c r="R23" s="40"/>
+      <c r="S23" s="38">
+        <f ca="1">SUM(S8:S13)+SUM(S17:S21)</f>
+        <v>23079503.823178016</v>
+      </c>
+      <c r="T23" s="42">
+        <f ca="1">SUM(T8:T13)+SUM(T17:T21)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B25" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B26" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="13">
+        <f ca="1">Inputs!C19/SeriesA!N20</f>
+        <v>8.3861588870237789</v>
+      </c>
+      <c r="T26" s="3"/>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B27" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="11">
+        <f>Inputs!C19+Inputs!C20</f>
+        <v>180000000</v>
+      </c>
+      <c r="T27" s="3"/>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B28" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="12">
+        <f ca="1">SeriesA!N23</f>
+        <v>4.1246318559836945</v>
+      </c>
+      <c r="T28" s="3"/>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="12">
+        <f ca="1">SeriesA!N24</f>
+        <v>4.9495582271804333</v>
+      </c>
+      <c r="T29" s="3"/>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>